<commit_message>
Add project.nuget.cache file with package dependencies and metadata
</commit_message>
<xml_diff>
--- a/project docs/urbanhub_Db.xlsx
+++ b/project docs/urbanhub_Db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aiubedu60714-my.sharepoint.com/personal/23-50139-1_student_aiub_edu/Documents/uni/10 sem/A .NET/Urbanhub/project docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{7CAAB226-5146-44EB-A7A4-A8190A84AC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEB17D2A-9CF0-4C35-9D92-00C7821E012C}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{7CAAB226-5146-44EB-A7A4-A8190A84AC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADB36F88-5506-45EA-979F-036E0F50C879}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E6CBEEEF-7371-4B4C-B4C6-722456DC993D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E6CBEEEF-7371-4B4C-B4C6-722456DC993D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="99">
   <si>
     <t>auth</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>oid(fk)</t>
+  </si>
+  <si>
+    <t>Owner</t>
   </si>
 </sst>
 </file>
@@ -1435,7 +1438,7 @@
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
       <c r="C28" s="1" t="s">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="5"/>

</xml_diff>